<commit_message>
Add SciTOX rebuild demo and agent prompts
</commit_message>
<xml_diff>
--- a/outputs/scitox_product_data/Product_Data_Requirements.xlsx
+++ b/outputs/scitox_product_data/Product_Data_Requirements.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Data" sheetId="1" r:id="Raf44784dea3d4a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R36b856fa3a8d4aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R900a90c27cd04740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Data" sheetId="1" r:id="R2567cab8e44547f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R6f131d36fee34eae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R5872a0d3e12f4ecc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2357,7 +2357,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c6a38190e0f44c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf330679579c440fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2681,7 +2681,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racf2257088f54927"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4457d23953de449e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>